<commit_message>
Add some options for specialized use of the MSAT.
</commit_message>
<xml_diff>
--- a/data_raw/MSAT_dict.xlsx
+++ b/data_raw/MSAT_dict.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hake Home PC\Dropbox\Uni Oldenburg\#3 - RStudio dateien\#4 - MSAT - main test R script\MSA\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFFD0BDF-6BC8-406D-BF3C-6F11D19ACE29}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C42DCF29-0AFC-4990-ACD2-C949A8FC0298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="30195" yWindow="300" windowWidth="14190" windowHeight="14565" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-1785" windowWidth="38640" windowHeight="20865" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="EDT" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="81">
   <si>
     <t>key</t>
   </si>
@@ -55,18 +55,6 @@
     <t>FEEDBACK</t>
   </si>
   <si>
-    <t>ANGRIER</t>
-  </si>
-  <si>
-    <t>HAPPIER</t>
-  </si>
-  <si>
-    <t>TENDER</t>
-  </si>
-  <si>
-    <t>SADDER</t>
-  </si>
-  <si>
     <t>ENTER_ID</t>
   </si>
   <si>
@@ -94,27 +82,12 @@
     <t>Frage {{num_question}} von {{test_length}}</t>
   </si>
   <si>
-    <t>Dein Browser unterstützt kein Audio. Dieser Test funktioniert nicht ohne Audio, sorry!</t>
-  </si>
-  <si>
     <t>Bitte eine Option auswählen.</t>
   </si>
   <si>
     <t>Herzlichen Glückwunsch!</t>
   </si>
   <si>
-    <t>wütender</t>
-  </si>
-  <si>
-    <t>fröhlicher</t>
-  </si>
-  <si>
-    <t>zärtlicher</t>
-  </si>
-  <si>
-    <t>trauriger</t>
-  </si>
-  <si>
     <t>Bitte gib Deine ID ein</t>
   </si>
   <si>
@@ -136,27 +109,12 @@
     <t>Question {{num_question}} out of {{test_length}}</t>
   </si>
   <si>
-    <t>Your browser doesn't support audio. This test won't work without audio, sorry!</t>
-  </si>
-  <si>
     <t>Please select one option.</t>
   </si>
   <si>
     <t>Congratulations!</t>
   </si>
   <si>
-    <t>angrier</t>
-  </si>
-  <si>
-    <t>happier</t>
-  </si>
-  <si>
-    <t>more tender</t>
-  </si>
-  <si>
-    <t>sadder</t>
-  </si>
-  <si>
     <t>Please enter your ID.</t>
   </si>
   <si>
@@ -175,45 +133,146 @@
     <t>Score</t>
   </si>
   <si>
-    <t>Willkommen zum MSAT</t>
-  </si>
-  <si>
-    <t>Welcome to the MSAT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bitte wählen Sie (Ja) oder (Nein), je nachdem, ob Sie das einzelne Zielinstrument in der Mixtur gehört haben oder nicht. Wenn Sie sich nicht sicher sind, nehmen Sie die Antwort, die Sie für richtig halten. </t>
-  </si>
-  <si>
     <t>Du hast den Test zur musikalischen Szenenanalyse erfolgreich beendet.</t>
   </si>
   <si>
     <t>Musikalische Szenenanalyse Test</t>
   </si>
   <si>
-    <t xml:space="preserve">In the experiment, you will be presented with various music excerpts. Each music excerpt consists of two parts. In the first part a single instrument (voice or bass) plays, in the second part a mixture of several instruments (mixture). 
+    <t>Musical Scene Analysis Test</t>
+  </si>
+  <si>
+    <t>You have completed the Musical Scene Analysis test.</t>
+  </si>
+  <si>
+    <t>Du hast **{{accuracy}} %** der Musikinstrumente richtig erkannt.</t>
+  </si>
+  <si>
+    <t>You recognized **{{accuracy}} %**  of the music excerpts correctly.</t>
+  </si>
+  <si>
+    <t>Willkommen zum Test zur Musikalischen Szenenanalysen (MSAT)</t>
+  </si>
+  <si>
+    <t>Welcome to the test for musical scene analysis (MSAT)</t>
+  </si>
+  <si>
+    <t>GOBACK</t>
+  </si>
+  <si>
+    <t>Gehe zurück</t>
+  </si>
+  <si>
+    <t>Go back</t>
+  </si>
+  <si>
+    <t>INSTRUCTIONS</t>
+  </si>
+  <si>
+    <t>SAMPLE1a</t>
+  </si>
+  <si>
+    <t>SAMPLE1b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In diesem Beispiel ist das Zielsintrument (Piano) in der Mixtur zu hören
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In diesem Beispiel ist das Zielsintrument (Hauptgesang) nicht in der Mixtur zu hören.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Here, the target instrument (piano) plays in the mixture. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Here, the target instrument (lead voice) does not play in the mixture. </t>
+  </si>
+  <si>
+    <t>PRACTICE1</t>
+  </si>
+  <si>
+    <t>PRACTICE2</t>
+  </si>
+  <si>
+    <t>TRANSITION</t>
+  </si>
+  <si>
+    <t>**{{feedback}}** \\ Klicke auf 'Zurück', um die Anweisungen erneut zu lesen und die Beispiele erneut zu versuchen, oder klicke auf 'Weiter', um zum  Haupttest zu gelangen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">**{{feedback}}** \\ Press ‘Go back’ to read the instructions and do the practice questions again, or press ‘Continue’ to continue to the main test. </t>
+  </si>
+  <si>
+    <t>INCORRECT</t>
+  </si>
+  <si>
+    <t>Falsch.</t>
+  </si>
+  <si>
+    <t>Incorrect.</t>
+  </si>
+  <si>
+    <t>CORRECT</t>
+  </si>
+  <si>
+    <t>Richtig!</t>
+  </si>
+  <si>
+    <t>Correct!</t>
+  </si>
+  <si>
+    <t>MAIN_INTRO</t>
+  </si>
+  <si>
+    <t>**{{feedback}}** \\ **Übungsfrage 2** \\ Bitte hören Sie sich den folgenden Clip an und wählen Sie aus, ob das Zielinstrument in der Instrumentenmixtur spielt.\\ Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> **{{feedback}}** \\ **Practice question 2** \\Please listen to the following clip and decide, whether the target plays in the mixture.\\  Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture.</t>
+  </si>
+  <si>
+    <t>**Übungsfrage 1** \\ Bitte hören Sie sich den folgenden Clip an und entscheiden Sie, ob das Zielinstrument in der Instrumentenmixtur spielte.\\ Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur"</t>
+  </si>
+  <si>
+    <t>**Practice question 1** \\ Please listen to the following clip and and decide, whether the target plays in the mixture.\\ Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture.</t>
+  </si>
+  <si>
+    <t>Nun geht es mit dem Haupttest los, in dem Ihre Antworten gespeichert werden. \\ Ab jetzt bekommen Sie keine Rückmeldung mehr. Viel Erfolg!</t>
+  </si>
+  <si>
+    <t>You are about to start the main test, where your results will be recorded. \\ You won't receive any feedback after individual questions. Good luck and have fun!</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Willkommen zum Test zur Musikalischen Szenenanalysen (MSAT)&lt;/h4&gt; In diesem Test werden Ihnen verschiedene Musikausschnitte dargeboten. Jeder Musikausschnitt besteht aus zwei Teilen. Im ersten Teil spielt ein einzelnes Instrument (Stimme, Bass, Gitarre der Klavier), im zweiten Teil eine Mischung aus mehreren Instrumenten (Mixtur). Ihre Aufgabe ist es zu entscheiden, ob das einzelne Zielinstrument in der Instrumentenmischung gespielt hat. 
+Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur".\\ Zuerst wirst du Beispiele hören und dann ein paar Übungsaufgaben machen.</t>
+  </si>
+  <si>
+    <t>&lt;h4&gt;Welcome to the test for musical scene analysis (MSAT)&lt;/h4&gt;  In the experiment, you will be presented with various music excerpts. Each music excerpt consists of two parts. In the first part a single instrument (lead voice, bass, guitar or piano) plays, in the second part a mixture of several instruments (mixture). 
 Your task is to decide whether the single target instrument played in the mixture of instruments. 
-Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture".
+Click "Yes" for "Yes - the target instrument played in the mixture" and "No" for "No - the target instrument did not play in the mixture".\\ First, you’ll hear some examples and do a few practice questions.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture. If you are not sure, take the answer you think is correct. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur". Wenn Sie sich nicht sicher sind, nehmen Sie die Antwort, die Sie für richtig halten. </t>
+  </si>
+  <si>
+    <t>Dein Browser unterstützt kein Audio. Dieser Test funktioniert nicht ohne Audio! Probieren Sie es bitte mit einem anderen Browser (bspw. Google Chrome).</t>
+  </si>
+  <si>
+    <t>Your browser doesn't support audio. This test won't work without audio, sorry! Pleas try using another Browser (e.g. Google Chrome).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the experiment, you will be presented with various music excerpts. Each music excerpt consists of two parts. In the first part a single instrument plays (lead voice, bass, guitar or piano), in the second part a mixture of several instruments (mixture). 
+Your task is to decide whether the single target instrument played in the mixture of instruments. 
+Click "1" for "Yes - the target instrument played in the mixture" and "2" for "No - the target instrument did not play in the mixture".
 </t>
   </si>
   <si>
-    <t>In diesem Test werden Ihnen verschiedene Musikausschnitte dargeboten. Jeder Musikausschnitt besteht aus zwei Teilen. Im ersten Teil spielt ein einzelnes Instrument (Stimme oder Bass), im zweiten Teil eine Mischung aus mehreren Instrumenten (Mixtur). 
+    <t>In diesem Test werden Ihnen verschiedene Musikausschnitte dargeboten. Jeder Musikausschnitt besteht aus zwei Teilen. Im ersten Teil spielt ein einzelnes Instrument (Stimme, Bass, Gitarre der Klavier), im zweiten Teil eine Mischung aus mehreren Instrumenten (Mixtur). 
 Ihre Aufgabe ist es zu entscheiden, ob das einzelne Zielinstrument in der Instrumentenmischung gespielt hat. 
-Klicken Sie auf "Ja" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "Nein" für "Nein - das Zielinstrument spielte nicht in der Mixtur".</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Please select (Yes) or (No) depending on whether you heard the single target instrument in the mixture or not. If you are not sure, take the answer you think is correct. </t>
-  </si>
-  <si>
-    <t>Musical Scene Analysis Test</t>
-  </si>
-  <si>
-    <t>You have completed the Musical Scene Analysis test.</t>
-  </si>
-  <si>
-    <t>Du hast **{{accuracy}} %** der Musikinstrumente richtig erkannt.</t>
-  </si>
-  <si>
-    <t>You recognized **{{accuracy}} %**  of the music excerpts correctly.</t>
+Klicken Sie auf "1" für "Ja - das Zielinstrument spielte in der Mixtur" und auf "2" für "Nein - das Zielinstrument spielte nicht in der Mixtur".</t>
   </si>
 </sst>
 </file>
@@ -249,11 +308,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -629,11 +700,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.5703125" customWidth="1"/>
     <col min="2" max="2" width="112.140625" customWidth="1"/>
+    <col min="3" max="3" width="100.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -647,26 +719,26 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -674,10 +746,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -685,10 +757,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -696,10 +768,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -707,10 +779,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -718,10 +790,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -729,10 +801,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -740,10 +812,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -751,10 +823,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>42</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -762,10 +834,10 @@
         <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -773,10 +845,10 @@
         <v>14</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C13" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -784,10 +856,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -795,10 +867,10 @@
         <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -806,10 +878,10 @@
         <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -817,54 +889,120 @@
         <v>18</v>
       </c>
       <c r="B17" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="90" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C17" t="s">
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" t="s">
-        <v>55</v>
-      </c>
-      <c r="C18" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>20</v>
-      </c>
-      <c r="B19" t="s">
-        <v>34</v>
-      </c>
-      <c r="C19" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" t="s">
-        <v>35</v>
-      </c>
-      <c r="C20" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" t="s">
-        <v>50</v>
+      <c r="B25" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>